<commit_message>
fix(v4): clarify final results, trace parameters and enforce rounded market cap
</commit_message>
<xml_diff>
--- a/Entrega-2/v4/demo/consolidated/consolidated_final.xlsx
+++ b/Entrega-2/v4/demo/consolidated/consolidated_final.xlsx
@@ -3,8 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookProtection workbookPassword="FE27" lockStructure="1"/>
   <sheets>
-    <sheet name="Final" sheetId="1" ns1:id="R83a49782582e4b9d"/>
-    <sheet name="Budgets" sheetId="2" ns1:id="Ra35e352b8a2d4654"/>
+    <sheet name="Final" sheetId="1" ns1:id="R442d3f7e2dc4453c"/>
+    <sheet name="Budgets" sheetId="2" ns1:id="Rc67f2bc32d3644d1"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,25 +430,25 @@
         <v>Market_Increase_Pct</v>
       </c>
       <c r="AB1" s="8" t="str">
-        <v>New_Salary</v>
+        <v>Proposed Salary</v>
       </c>
       <c r="AC1" s="8" t="str">
-        <v>Total_Increase_Pct</v>
+        <v>Proposed Increase %</v>
       </c>
       <c r="AD1" s="8" t="str">
-        <v>Final_Compa_Ratio</v>
+        <v>Proposed Compa Ratio</v>
       </c>
       <c r="AE1" s="8" t="str">
-        <v>Discretionary_Adjustment_Pct</v>
+        <v>Discretionary Adjustment %</v>
       </c>
       <c r="AF1" s="8" t="str">
-        <v>Final_Increase_Pct</v>
+        <v>Final Increase %</v>
       </c>
       <c r="AG1" s="8" t="str">
-        <v>Final_Salary</v>
+        <v>Final Salary</v>
       </c>
       <c r="AH1" s="8" t="str">
-        <v>Human_Final_Compa_Ratio</v>
+        <v>Final Compa Ratio</v>
       </c>
       <c r="AI1" s="8" t="str">
         <v>Human_Modified</v>

</xml_diff>